<commit_message>
More fixes for updating pivot cache source where field names has changed
</commit_message>
<xml_diff>
--- a/src/EPPlusTest/Workbooks/PivotTableRefreshFields.xlsx
+++ b/src/EPPlusTest/Workbooks/PivotTableRefreshFields.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\kod\EPPlusSoftware\EPPlus\src\EPPlusTest\Workbooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B82E2D31-DF70-4F8D-80A3-48217BF46D16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AE3E8CA-EEF2-4485-ABA1-763210D60BC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3510" yWindow="3510" windowWidth="57585" windowHeight="15345" activeTab="1" xr2:uid="{84C3C679-CD18-446A-BF71-AEC7DFD120C7}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="77040" windowHeight="21120" xr2:uid="{84C3C679-CD18-446A-BF71-AEC7DFD120C7}"/>
   </bookViews>
   <sheets>
     <sheet name="PivotSource" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,8 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="1" r:id="rId3"/>
+    <pivotCache cacheId="0" r:id="rId3"/>
+    <pivotCache cacheId="1" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="21">
   <si>
     <t>Id 1</t>
   </si>
@@ -83,12 +84,33 @@
   <si>
     <t>Id 2-new</t>
   </si>
+  <si>
+    <t>Count of 5</t>
+  </si>
+  <si>
+    <t>Text Three</t>
+  </si>
+  <si>
+    <t>Text Two</t>
+  </si>
+  <si>
+    <t>Code Five</t>
+  </si>
+  <si>
+    <t>Id Two-new</t>
+  </si>
+  <si>
+    <t>Five</t>
+  </si>
+  <si>
+    <t>Sum of test 3</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -102,16 +124,30 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor theme="4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -119,31 +155,71 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </right>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="2">
     <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFFF00"/>
-        </patternFill>
-      </fill>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
+        <b/>
         <i val="0"/>
         <strike val="0"/>
         <condense val="0"/>
@@ -153,25 +229,15 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
-        <color rgb="FF9C0006"/>
+        <color theme="0"/>
         <name val="Aptos Narrow"/>
         <family val="2"/>
         <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <fgColor indexed="65"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
         </patternFill>
       </fill>
     </dxf>
@@ -212,13 +278,35 @@
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="0.19688460138148489" maxValue="0.91550901170969556"/>
     </cacheField>
     <cacheField name="Text 3" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="5.7705468643579394E-2" maxValue="0.61848700428443393"/>
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="5.7705468643579394E-2" maxValue="0.61848700428443393" count="10">
+        <n v="0.13340413190495237"/>
+        <n v="0.30388423954630883"/>
+        <n v="0.60115544026098999"/>
+        <n v="0.61848700428443393"/>
+        <n v="0.4456171505246449"/>
+        <n v="5.7705468643579394E-2"/>
+        <n v="0.54949022232860489"/>
+        <n v="0.41381317840619092"/>
+        <n v="0.12700755913005879"/>
+        <n v="0.32445954533835186"/>
+      </sharedItems>
     </cacheField>
     <cacheField name="Text 2" numFmtId="0">
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="1.9400112590848728E-2" maxValue="0.99461144635169618"/>
     </cacheField>
     <cacheField name="Code 5" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="1.7695902902192806E-3" maxValue="0.92750814645224633"/>
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="1.7695902902192806E-3" maxValue="0.92750814645224633" count="10">
+        <n v="0.11299281224136282"/>
+        <n v="0.35663337324104227"/>
+        <n v="0.53942394424824758"/>
+        <n v="0.76106209391242419"/>
+        <n v="1.7695902902192806E-3"/>
+        <n v="0.92750814645224633"/>
+        <n v="0.15588152838397162"/>
+        <n v="0.33747648451066592"/>
+        <n v="6.9324790915765044E-2"/>
+        <n v="0.26829478472888124"/>
+      </sharedItems>
     </cacheField>
     <cacheField name="Id 1" numFmtId="0">
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="4.8454653904772327E-2" maxValue="0.80046306693405822" count="10">
@@ -260,14 +348,65 @@
 </pivotCacheDefinition>
 </file>
 
+<file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Janne" refreshedDate="45789.456288310183" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="11" xr:uid="{7EECEDCA-4542-4751-94E5-581ABE35EE8D}">
+  <cacheSource type="worksheet">
+    <worksheetSource name="Table224"/>
+  </cacheSource>
+  <cacheFields count="7">
+    <cacheField name="Id 2-new" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="0.25869945923185078" maxValue="0.90047506962074264"/>
+    </cacheField>
+    <cacheField name="Text 3" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="5.7705468643579394E-2" maxValue="0.61848700428443393"/>
+    </cacheField>
+    <cacheField name="Text 2" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="1.9400112590848728E-2" maxValue="0.99461144635169618"/>
+    </cacheField>
+    <cacheField name="Code 5" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="1.7695902902192806E-3" maxValue="0.92750814645224633"/>
+    </cacheField>
+    <cacheField name="Id 1" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="0.18873433406805584" maxValue="0.68547634721449247" count="10">
+        <n v="0.52825740988302194"/>
+        <n v="0.53076105377807759"/>
+        <n v="0.36864262914755841"/>
+        <n v="0.66295431661132742"/>
+        <n v="0.64905416145984174"/>
+        <n v="0.18873433406805584"/>
+        <n v="0.68547634721449247"/>
+        <n v="0.42934753902516243"/>
+        <n v="0.23708285003021579"/>
+        <n v="0.45226946132133428"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="5" numFmtId="0">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="4.8454653904772327E-2" maxValue="0.80046306693405822"/>
+    </cacheField>
+    <cacheField name="test 3" numFmtId="0">
+      <sharedItems count="3">
+        <s v="Text 1"/>
+        <s v="Text 2"/>
+        <s v="Text 3"/>
+      </sharedItems>
+    </cacheField>
+  </cacheFields>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
 <file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="11">
   <r>
     <x v="0"/>
     <n v="0.37777901065478803"/>
-    <n v="0.13340413190495237"/>
+    <x v="0"/>
     <n v="0.93167226865226405"/>
-    <n v="0.11299281224136282"/>
+    <x v="0"/>
     <x v="0"/>
     <s v="Text 1"/>
     <x v="0"/>
@@ -275,9 +414,9 @@
   <r>
     <x v="1"/>
     <n v="0.89791954931470097"/>
-    <n v="0.30388423954630883"/>
+    <x v="1"/>
     <n v="1.9400112590848728E-2"/>
-    <n v="0.35663337324104227"/>
+    <x v="1"/>
     <x v="1"/>
     <s v="Text 2"/>
     <x v="1"/>
@@ -285,9 +424,9 @@
   <r>
     <x v="2"/>
     <n v="0.54897468230100133"/>
-    <n v="0.60115544026098999"/>
+    <x v="2"/>
     <n v="0.80637778206434629"/>
-    <n v="0.53942394424824758"/>
+    <x v="2"/>
     <x v="2"/>
     <s v="Text 3"/>
     <x v="2"/>
@@ -295,9 +434,9 @@
   <r>
     <x v="3"/>
     <n v="0.19688460138148489"/>
-    <n v="0.61848700428443393"/>
+    <x v="3"/>
     <n v="0.23409291564020496"/>
-    <n v="0.76106209391242419"/>
+    <x v="3"/>
     <x v="3"/>
     <s v="Text 1"/>
     <x v="3"/>
@@ -305,9 +444,9 @@
   <r>
     <x v="4"/>
     <n v="0.6956516588377355"/>
-    <n v="0.4456171505246449"/>
+    <x v="4"/>
     <n v="0.99461144635169618"/>
-    <n v="1.7695902902192806E-3"/>
+    <x v="4"/>
     <x v="4"/>
     <s v="Text 2"/>
     <x v="4"/>
@@ -315,9 +454,9 @@
   <r>
     <x v="5"/>
     <n v="0.91550901170969556"/>
-    <n v="5.7705468643579394E-2"/>
+    <x v="5"/>
     <n v="0.21306041435280476"/>
-    <n v="0.92750814645224633"/>
+    <x v="5"/>
     <x v="5"/>
     <s v="Text 1"/>
     <x v="5"/>
@@ -325,9 +464,9 @@
   <r>
     <x v="6"/>
     <n v="0.21822830924232139"/>
-    <n v="0.54949022232860489"/>
+    <x v="6"/>
     <n v="0.37586842832109557"/>
-    <n v="0.15588152838397162"/>
+    <x v="6"/>
     <x v="6"/>
     <s v="Text 1"/>
     <x v="6"/>
@@ -335,9 +474,9 @@
   <r>
     <x v="7"/>
     <n v="0.48523760941160798"/>
-    <n v="0.41381317840619092"/>
+    <x v="7"/>
     <n v="0.23990691494196548"/>
-    <n v="0.33747648451066592"/>
+    <x v="7"/>
     <x v="7"/>
     <s v="Text 2"/>
     <x v="7"/>
@@ -345,9 +484,9 @@
   <r>
     <x v="8"/>
     <n v="0.62456224048693332"/>
-    <n v="0.12700755913005879"/>
+    <x v="8"/>
     <n v="9.8357132323889651E-2"/>
-    <n v="6.9324790915765044E-2"/>
+    <x v="8"/>
     <x v="8"/>
     <s v="Text 3"/>
     <x v="8"/>
@@ -355,9 +494,9 @@
   <r>
     <x v="9"/>
     <n v="0.67767971164282126"/>
-    <n v="0.32445954533835186"/>
+    <x v="9"/>
     <n v="0.36328565968295456"/>
-    <n v="0.26829478472888124"/>
+    <x v="9"/>
     <x v="9"/>
     <s v="Text 2"/>
     <x v="9"/>
@@ -365,9 +504,9 @@
   <r>
     <x v="9"/>
     <n v="0.67767971164282126"/>
-    <n v="0.32445954533835186"/>
+    <x v="9"/>
     <n v="0.36328565968295456"/>
-    <n v="0.26829478472888124"/>
+    <x v="9"/>
     <x v="9"/>
     <s v="Text 3"/>
     <x v="9"/>
@@ -375,29 +514,133 @@
 </pivotCacheRecords>
 </file>
 
+<file path=xl/pivotCache/pivotCacheRecords2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="11">
+  <r>
+    <n v="0.49965214247168532"/>
+    <n v="0.13340413190495237"/>
+    <n v="0.93167226865226405"/>
+    <n v="0.11299281224136282"/>
+    <x v="0"/>
+    <n v="0.75854847124746105"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <n v="0.69052391867761753"/>
+    <n v="0.30388423954630883"/>
+    <n v="1.9400112590848728E-2"/>
+    <n v="0.35663337324104227"/>
+    <x v="1"/>
+    <n v="0.47358850809372832"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <n v="0.41372134280827666"/>
+    <n v="0.60115544026098999"/>
+    <n v="0.80637778206434629"/>
+    <n v="0.53942394424824758"/>
+    <x v="2"/>
+    <n v="0.80046306693405822"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <n v="0.90047506962074264"/>
+    <n v="0.61848700428443393"/>
+    <n v="0.23409291564020496"/>
+    <n v="0.76106209391242419"/>
+    <x v="3"/>
+    <n v="0.76916581804686701"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <n v="0.73258527600204193"/>
+    <n v="0.4456171505246449"/>
+    <n v="0.99461144635169618"/>
+    <n v="1.7695902902192806E-3"/>
+    <x v="4"/>
+    <n v="0.34534484287961087"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <n v="0.32828173765972979"/>
+    <n v="5.7705468643579394E-2"/>
+    <n v="0.21306041435280476"/>
+    <n v="0.92750814645224633"/>
+    <x v="5"/>
+    <n v="0.18907147041048855"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <n v="0.42256856514005547"/>
+    <n v="0.54949022232860489"/>
+    <n v="0.37586842832109557"/>
+    <n v="0.15588152838397162"/>
+    <x v="6"/>
+    <n v="4.8454653904772327E-2"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <n v="0.25869945923185078"/>
+    <n v="0.41381317840619092"/>
+    <n v="0.23990691494196548"/>
+    <n v="0.33747648451066592"/>
+    <x v="7"/>
+    <n v="0.46566382181943422"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <n v="0.69522506560877662"/>
+    <n v="0.12700755913005879"/>
+    <n v="9.8357132323889651E-2"/>
+    <n v="6.9324790915765044E-2"/>
+    <x v="8"/>
+    <n v="9.5740302083714868E-2"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <n v="0.86989023905705309"/>
+    <n v="0.32445954533835186"/>
+    <n v="0.36328565968295456"/>
+    <n v="0.26829478472888124"/>
+    <x v="9"/>
+    <n v="0.19384266692417795"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <n v="0.86989023905705309"/>
+    <n v="0.32445954533835186"/>
+    <n v="0.36328565968295456"/>
+    <n v="0.26829478472888124"/>
+    <x v="9"/>
+    <n v="0.19384266692417795"/>
+    <x v="2"/>
+  </r>
+</pivotCacheRecords>
+</file>
+
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A2E54A3F-70A5-4381-BDBA-D18068B4FFF9}" name="PivotTable2" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0">
-  <location ref="A23:L35" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{72E042A0-B457-489A-AD90-45836115D8E9}" name="PivotTable3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="W3:AH5" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="8">
-    <pivotField axis="axisRow" showAll="0">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisPage" showAll="0">
       <items count="11">
         <item x="5"/>
         <item x="8"/>
-        <item x="2"/>
-        <item x="7"/>
-        <item x="9"/>
         <item x="0"/>
         <item x="1"/>
+        <item x="9"/>
+        <item x="7"/>
         <item x="4"/>
+        <item x="6"/>
+        <item x="2"/>
         <item x="3"/>
-        <item x="6"/>
         <item t="default"/>
       </items>
     </pivotField>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
     <pivotField axis="axisCol" showAll="0">
       <items count="11">
         <item x="6"/>
@@ -414,59 +657,10 @@
       </items>
     </pivotField>
     <pivotField showAll="0"/>
-    <pivotField axis="axisPage" showAll="0">
-      <items count="11">
-        <item x="7"/>
-        <item x="5"/>
-        <item x="2"/>
-        <item x="6"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="8"/>
-        <item x="4"/>
-        <item x="9"/>
-        <item x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
+    <pivotField dataField="1" showAll="0"/>
   </pivotFields>
-  <rowFields count="1">
-    <field x="0"/>
-  </rowFields>
-  <rowItems count="11">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="8"/>
-    </i>
-    <i>
-      <x v="9"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
+  <rowItems count="1">
+    <i/>
   </rowItems>
   <colFields count="1">
     <field x="5"/>
@@ -507,10 +701,251 @@
     </i>
   </colItems>
   <pageFields count="1">
-    <pageField fld="7" hier="-1"/>
+    <pageField fld="2" hier="-1"/>
   </pageFields>
   <dataFields count="1">
-    <dataField name="Sum of Code 5" fld="4" baseField="0" baseItem="0"/>
+    <dataField name="Sum of test 3" fld="7" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{4D80E5F4-4078-4B61-BA24-862631189B98}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A3:L15" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
+  <pivotFields count="8">
+    <pivotField axis="axisPage" showAll="0">
+      <items count="11">
+        <item x="5"/>
+        <item x="8"/>
+        <item x="2"/>
+        <item x="7"/>
+        <item x="9"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item x="6"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="11">
+        <item x="5"/>
+        <item x="8"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="9"/>
+        <item x="7"/>
+        <item x="4"/>
+        <item x="6"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="11">
+        <item x="4"/>
+        <item x="8"/>
+        <item x="0"/>
+        <item x="6"/>
+        <item x="9"/>
+        <item x="7"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="5"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="4"/>
+  </rowFields>
+  <rowItems count="11">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="2"/>
+  </colFields>
+  <colItems count="11">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <pageFields count="1">
+    <pageField fld="0" hier="-1"/>
+  </pageFields>
+  <dataFields count="1">
+    <dataField name="Count of 5" fld="6" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2148893D-99A8-4442-9F9C-31B89BC31B70}" name="PivotTable2" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" multipleFieldFilters="0">
+  <location ref="A23:L25" firstHeaderRow="1" firstDataRow="2" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
+  <pivotFields count="7">
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField axis="axisCol" showAll="0">
+      <items count="11">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisPage" showAll="0">
+      <items count="4">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowItems count="1">
+    <i/>
+  </rowItems>
+  <colFields count="1">
+    <field x="4"/>
+  </colFields>
+  <colItems count="11">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </colItems>
+  <pageFields count="1">
+    <pageField fld="6" hier="-1"/>
+  </pageFields>
+  <dataFields count="1">
+    <dataField name="Sum of Code 5" fld="3" baseField="0" baseItem="0"/>
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
@@ -552,6 +987,22 @@
     <tableColumn id="1" xr3:uid="{F613FDAE-6145-4FC2-B2CA-C20EE97CFFA7}" name="Id 1"/>
     <tableColumn id="7" xr3:uid="{C9FBD844-7D56-4AFE-B626-CE2B963999D1}" name="5"/>
     <tableColumn id="8" xr3:uid="{4377B515-8E5F-4D87-8FFA-63B94BD58453}" name="test 3"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{6732FC2A-DFA4-4923-86E8-D322900ACDC3}" name="Table224" displayName="Table224" ref="A15:G26" totalsRowShown="0" headerRowDxfId="1" headerRowBorderDxfId="0">
+  <autoFilter ref="A15:G26" xr:uid="{6732FC2A-DFA4-4923-86E8-D322900ACDC3}"/>
+  <tableColumns count="7">
+    <tableColumn id="8" xr3:uid="{E6386FF4-123D-49AE-B96E-EF86C42C89AA}" name="test 3"/>
+    <tableColumn id="3" xr3:uid="{86A81C1D-0E22-4984-95D2-070CB73E765D}" name="Text Three"/>
+    <tableColumn id="4" xr3:uid="{B69A2FFE-89D3-41F1-9DDE-ADD6D34C99F5}" name="Text Two"/>
+    <tableColumn id="6" xr3:uid="{05A92E7A-6587-4AD1-A7DA-A79DB70AEA03}" name="Code Five"/>
+    <tableColumn id="2" xr3:uid="{FB5B3635-F751-4269-8F99-54297F35F834}" name="Id Two-new"/>
+    <tableColumn id="1" xr3:uid="{85961D51-4DC2-43BD-8F6A-A436D48A9D7D}" name="Id 1"/>
+    <tableColumn id="7" xr3:uid="{F8D260F2-7D43-4A69-8E37-B18E37DE7408}" name="Five"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -874,10 +1325,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{928AE3D7-705D-4E0E-94EA-433A1B141953}">
-  <dimension ref="A1:P12"/>
+  <dimension ref="A1:P26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="8" max="8" width="9.42578125" customWidth="1"/>
+    <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12" bestFit="1" customWidth="1"/>
+    <col min="10" max="14" width="12" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="5.85546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
@@ -1444,19 +1905,296 @@
         <v>0.86989023905705309</v>
       </c>
     </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="G15" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>0.49965214247168532</v>
+      </c>
+      <c r="B16">
+        <v>0.13340413190495237</v>
+      </c>
+      <c r="C16">
+        <v>0.93167226865226405</v>
+      </c>
+      <c r="D16">
+        <v>0.11299281224136282</v>
+      </c>
+      <c r="E16">
+        <v>0.52825740988302194</v>
+      </c>
+      <c r="F16">
+        <v>0.75854847124746105</v>
+      </c>
+      <c r="G16" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>0.69052391867761753</v>
+      </c>
+      <c r="B17">
+        <v>0.30388423954630883</v>
+      </c>
+      <c r="C17">
+        <v>1.9400112590848728E-2</v>
+      </c>
+      <c r="D17">
+        <v>0.35663337324104227</v>
+      </c>
+      <c r="E17">
+        <v>0.53076105377807759</v>
+      </c>
+      <c r="F17">
+        <v>0.47358850809372832</v>
+      </c>
+      <c r="G17" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>0.41372134280827666</v>
+      </c>
+      <c r="B18">
+        <v>0.60115544026098999</v>
+      </c>
+      <c r="C18">
+        <v>0.80637778206434629</v>
+      </c>
+      <c r="D18">
+        <v>0.53942394424824758</v>
+      </c>
+      <c r="E18">
+        <v>0.36864262914755841</v>
+      </c>
+      <c r="F18">
+        <v>0.80046306693405822</v>
+      </c>
+      <c r="G18" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>0.90047506962074264</v>
+      </c>
+      <c r="B19">
+        <v>0.61848700428443393</v>
+      </c>
+      <c r="C19">
+        <v>0.23409291564020496</v>
+      </c>
+      <c r="D19">
+        <v>0.76106209391242419</v>
+      </c>
+      <c r="E19">
+        <v>0.66295431661132742</v>
+      </c>
+      <c r="F19">
+        <v>0.76916581804686701</v>
+      </c>
+      <c r="G19" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>0.73258527600204193</v>
+      </c>
+      <c r="B20">
+        <v>0.4456171505246449</v>
+      </c>
+      <c r="C20">
+        <v>0.99461144635169618</v>
+      </c>
+      <c r="D20">
+        <v>1.7695902902192806E-3</v>
+      </c>
+      <c r="E20">
+        <v>0.64905416145984174</v>
+      </c>
+      <c r="F20">
+        <v>0.34534484287961087</v>
+      </c>
+      <c r="G20" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>0.32828173765972979</v>
+      </c>
+      <c r="B21">
+        <v>5.7705468643579394E-2</v>
+      </c>
+      <c r="C21">
+        <v>0.21306041435280476</v>
+      </c>
+      <c r="D21">
+        <v>0.92750814645224633</v>
+      </c>
+      <c r="E21">
+        <v>0.18873433406805584</v>
+      </c>
+      <c r="F21">
+        <v>0.18907147041048855</v>
+      </c>
+      <c r="G21" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>0.42256856514005547</v>
+      </c>
+      <c r="B22">
+        <v>0.54949022232860489</v>
+      </c>
+      <c r="C22">
+        <v>0.37586842832109557</v>
+      </c>
+      <c r="D22">
+        <v>0.15588152838397162</v>
+      </c>
+      <c r="E22">
+        <v>0.68547634721449247</v>
+      </c>
+      <c r="F22">
+        <v>4.8454653904772327E-2</v>
+      </c>
+      <c r="G22" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>0.25869945923185078</v>
+      </c>
+      <c r="B23">
+        <v>0.41381317840619092</v>
+      </c>
+      <c r="C23">
+        <v>0.23990691494196548</v>
+      </c>
+      <c r="D23">
+        <v>0.33747648451066592</v>
+      </c>
+      <c r="E23">
+        <v>0.42934753902516243</v>
+      </c>
+      <c r="F23">
+        <v>0.46566382181943422</v>
+      </c>
+      <c r="G23" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>0.69522506560877662</v>
+      </c>
+      <c r="B24">
+        <v>0.12700755913005879</v>
+      </c>
+      <c r="C24">
+        <v>9.8357132323889651E-2</v>
+      </c>
+      <c r="D24">
+        <v>6.9324790915765044E-2</v>
+      </c>
+      <c r="E24">
+        <v>0.23708285003021579</v>
+      </c>
+      <c r="F24">
+        <v>9.5740302083714868E-2</v>
+      </c>
+      <c r="G24" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>0.86989023905705309</v>
+      </c>
+      <c r="B25">
+        <v>0.32445954533835186</v>
+      </c>
+      <c r="C25">
+        <v>0.36328565968295456</v>
+      </c>
+      <c r="D25">
+        <v>0.26829478472888124</v>
+      </c>
+      <c r="E25">
+        <v>0.45226946132133428</v>
+      </c>
+      <c r="F25">
+        <v>0.19384266692417795</v>
+      </c>
+      <c r="G25" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>0.86989023905705309</v>
+      </c>
+      <c r="B26">
+        <v>0.32445954533835186</v>
+      </c>
+      <c r="C26">
+        <v>0.36328565968295456</v>
+      </c>
+      <c r="D26">
+        <v>0.26829478472888124</v>
+      </c>
+      <c r="E26">
+        <v>0.45226946132133428</v>
+      </c>
+      <c r="F26">
+        <v>0.19384266692417795</v>
+      </c>
+      <c r="G26" t="s">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="2">
+  <tableParts count="3">
     <tablePart r:id="rId1"/>
     <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0220B4B5-8E96-4CAE-A664-9E90EC14A3D0}">
-  <dimension ref="A21:L35"/>
+  <dimension ref="A1:AH25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.140625" bestFit="1" customWidth="1"/>
@@ -1472,9 +2210,291 @@
     <col min="20" max="20" width="12" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="13.140625" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="25" max="34" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="1" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>7</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="X1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="X3" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4">
+        <v>5.7705468643579394E-2</v>
+      </c>
+      <c r="C4">
+        <v>0.12700755913005879</v>
+      </c>
+      <c r="D4">
+        <v>0.13340413190495237</v>
+      </c>
+      <c r="E4">
+        <v>0.30388423954630883</v>
+      </c>
+      <c r="F4">
+        <v>0.32445954533835186</v>
+      </c>
+      <c r="G4">
+        <v>0.41381317840619092</v>
+      </c>
+      <c r="H4">
+        <v>0.4456171505246449</v>
+      </c>
+      <c r="I4">
+        <v>0.54949022232860489</v>
+      </c>
+      <c r="J4">
+        <v>0.60115544026098999</v>
+      </c>
+      <c r="K4">
+        <v>0.61848700428443393</v>
+      </c>
+      <c r="L4" t="s">
+        <v>9</v>
+      </c>
+      <c r="X4">
+        <v>4.8454653904772327E-2</v>
+      </c>
+      <c r="Y4">
+        <v>9.5740302083714868E-2</v>
+      </c>
+      <c r="Z4">
+        <v>0.18907147041048855</v>
+      </c>
+      <c r="AA4">
+        <v>0.19384266692417795</v>
+      </c>
+      <c r="AB4">
+        <v>0.34534484287961087</v>
+      </c>
+      <c r="AC4">
+        <v>0.46566382181943422</v>
+      </c>
+      <c r="AD4">
+        <v>0.47358850809372832</v>
+      </c>
+      <c r="AE4">
+        <v>0.75854847124746105</v>
+      </c>
+      <c r="AF4">
+        <v>0.76916581804686701</v>
+      </c>
+      <c r="AG4">
+        <v>0.80046306693405822</v>
+      </c>
+      <c r="AH4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A5" s="2">
+        <v>1.7695902902192806E-3</v>
+      </c>
+      <c r="H5">
+        <v>1</v>
+      </c>
+      <c r="L5">
+        <v>1</v>
+      </c>
+      <c r="W5" t="s">
+        <v>20</v>
+      </c>
+      <c r="X5">
+        <v>0.42256856514005547</v>
+      </c>
+      <c r="Y5">
+        <v>0.69522506560877662</v>
+      </c>
+      <c r="Z5">
+        <v>0.32828173765972979</v>
+      </c>
+      <c r="AA5">
+        <v>1.7397804781141062</v>
+      </c>
+      <c r="AB5">
+        <v>0.73258527600204193</v>
+      </c>
+      <c r="AC5">
+        <v>0.25869945923185078</v>
+      </c>
+      <c r="AD5">
+        <v>0.69052391867761753</v>
+      </c>
+      <c r="AE5">
+        <v>0.49965214247168532</v>
+      </c>
+      <c r="AF5">
+        <v>0.90047506962074264</v>
+      </c>
+      <c r="AG5">
+        <v>0.41372134280827666</v>
+      </c>
+      <c r="AH5">
+        <v>6.6815130553348823</v>
+      </c>
+    </row>
+    <row r="6" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A6" s="2">
+        <v>6.9324790915765044E-2</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="L6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A7" s="2">
+        <v>0.11299281224136282</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="L7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
+        <v>0.15588152838397162</v>
+      </c>
+      <c r="I8">
+        <v>1</v>
+      </c>
+      <c r="L8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A9" s="2">
+        <v>0.26829478472888124</v>
+      </c>
+      <c r="F9">
+        <v>2</v>
+      </c>
+      <c r="L9">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A10" s="2">
+        <v>0.33747648451066592</v>
+      </c>
+      <c r="G10">
+        <v>1</v>
+      </c>
+      <c r="L10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A11" s="2">
+        <v>0.35663337324104227</v>
+      </c>
+      <c r="E11">
+        <v>1</v>
+      </c>
+      <c r="L11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A12" s="2">
+        <v>0.53942394424824758</v>
+      </c>
+      <c r="J12">
+        <v>1</v>
+      </c>
+      <c r="L12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A13" s="2">
+        <v>0.76106209391242419</v>
+      </c>
+      <c r="K13">
+        <v>1</v>
+      </c>
+      <c r="L13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A14" s="2">
+        <v>0.92750814645224633</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="L14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15">
+        <v>1</v>
+      </c>
+      <c r="D15">
+        <v>1</v>
+      </c>
+      <c r="E15">
+        <v>1</v>
+      </c>
+      <c r="F15">
+        <v>2</v>
+      </c>
+      <c r="G15">
+        <v>1</v>
+      </c>
+      <c r="H15">
+        <v>1</v>
+      </c>
+      <c r="I15">
+        <v>1</v>
+      </c>
+      <c r="J15">
+        <v>1</v>
+      </c>
+      <c r="K15">
+        <v>1</v>
+      </c>
+      <c r="L15">
+        <v>11</v>
+      </c>
+    </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>6</v>
@@ -1484,197 +2504,81 @@
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
-        <v>12</v>
-      </c>
       <c r="B23" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="s">
-        <v>10</v>
-      </c>
       <c r="B24">
-        <v>4.8454653904772327E-2</v>
+        <v>0.52825740988302194</v>
       </c>
       <c r="C24">
-        <v>9.5740302083714868E-2</v>
+        <v>0.53076105377807759</v>
       </c>
       <c r="D24">
-        <v>0.18907147041048855</v>
+        <v>0.36864262914755841</v>
       </c>
       <c r="E24">
-        <v>0.19384266692417795</v>
+        <v>0.66295431661132742</v>
       </c>
       <c r="F24">
-        <v>0.34534484287961087</v>
+        <v>0.64905416145984174</v>
       </c>
       <c r="G24">
-        <v>0.46566382181943422</v>
+        <v>0.18873433406805584</v>
       </c>
       <c r="H24">
-        <v>0.47358850809372832</v>
+        <v>0.68547634721449247</v>
       </c>
       <c r="I24">
-        <v>0.75854847124746105</v>
+        <v>0.42934753902516243</v>
       </c>
       <c r="J24">
-        <v>0.76916581804686701</v>
+        <v>0.23708285003021579</v>
       </c>
       <c r="K24">
-        <v>0.80046306693405822</v>
+        <v>0.45226946132133428</v>
       </c>
       <c r="L24" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A25" s="2">
-        <v>0.18873433406805584</v>
+      <c r="A25" t="s">
+        <v>12</v>
+      </c>
+      <c r="B25">
+        <v>0.11299281224136282</v>
+      </c>
+      <c r="C25">
+        <v>0.35663337324104227</v>
       </c>
       <c r="D25">
+        <v>0.53942394424824758</v>
+      </c>
+      <c r="E25">
+        <v>0.76106209391242419</v>
+      </c>
+      <c r="F25">
+        <v>1.7695902902192806E-3</v>
+      </c>
+      <c r="G25">
         <v>0.92750814645224633</v>
       </c>
+      <c r="H25">
+        <v>0.15588152838397162</v>
+      </c>
+      <c r="I25">
+        <v>0.33747648451066592</v>
+      </c>
+      <c r="J25">
+        <v>6.9324790915765044E-2</v>
+      </c>
+      <c r="K25">
+        <v>0.53658956945776248</v>
+      </c>
       <c r="L25">
-        <v>0.92750814645224633</v>
-      </c>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A26" s="2">
-        <v>0.23708285003021579</v>
-      </c>
-      <c r="C26">
-        <v>6.9324790915765044E-2</v>
-      </c>
-      <c r="L26">
-        <v>6.9324790915765044E-2</v>
-      </c>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A27" s="2">
-        <v>0.36864262914755841</v>
-      </c>
-      <c r="K27">
-        <v>0.53942394424824758</v>
-      </c>
-      <c r="L27">
-        <v>0.53942394424824758</v>
-      </c>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A28" s="2">
-        <v>0.42934753902516243</v>
-      </c>
-      <c r="G28">
-        <v>0.33747648451066592</v>
-      </c>
-      <c r="L28">
-        <v>0.33747648451066592</v>
-      </c>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A29" s="2">
-        <v>0.45226946132133428</v>
-      </c>
-      <c r="E29">
-        <v>0.53658956945776248</v>
-      </c>
-      <c r="L29">
-        <v>0.53658956945776248</v>
-      </c>
-    </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A30" s="2">
-        <v>0.52825740988302194</v>
-      </c>
-      <c r="I30">
-        <v>0.11299281224136282</v>
-      </c>
-      <c r="L30">
-        <v>0.11299281224136282</v>
-      </c>
-    </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A31" s="2">
-        <v>0.53076105377807759</v>
-      </c>
-      <c r="H31">
-        <v>0.35663337324104227</v>
-      </c>
-      <c r="L31">
-        <v>0.35663337324104227</v>
-      </c>
-    </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A32" s="2">
-        <v>0.64905416145984174</v>
-      </c>
-      <c r="F32">
-        <v>1.7695902902192806E-3</v>
-      </c>
-      <c r="L32">
-        <v>1.7695902902192806E-3</v>
-      </c>
-    </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A33" s="2">
-        <v>0.66295431661132742</v>
-      </c>
-      <c r="J33">
-        <v>0.76106209391242419</v>
-      </c>
-      <c r="L33">
-        <v>0.76106209391242419</v>
-      </c>
-    </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A34" s="2">
-        <v>0.68547634721449247</v>
-      </c>
-      <c r="B34">
-        <v>0.15588152838397162</v>
-      </c>
-      <c r="L34">
-        <v>0.15588152838397162</v>
-      </c>
-    </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A35" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B35">
-        <v>0.15588152838397162</v>
-      </c>
-      <c r="C35">
-        <v>6.9324790915765044E-2</v>
-      </c>
-      <c r="D35">
-        <v>0.92750814645224633</v>
-      </c>
-      <c r="E35">
-        <v>0.53658956945776248</v>
-      </c>
-      <c r="F35">
-        <v>1.7695902902192806E-3</v>
-      </c>
-      <c r="G35">
-        <v>0.33747648451066592</v>
-      </c>
-      <c r="H35">
-        <v>0.35663337324104227</v>
-      </c>
-      <c r="I35">
-        <v>0.11299281224136282</v>
-      </c>
-      <c r="J35">
-        <v>0.76106209391242419</v>
-      </c>
-      <c r="K35">
-        <v>0.53942394424824758</v>
-      </c>
-      <c r="L35">
-        <v>3.7986623336537071</v>
+        <v>3.798662333653708</v>
       </c>
     </row>
   </sheetData>

</xml_diff>